<commit_message>
Group join api done and tested
</commit_message>
<xml_diff>
--- a/docs/Työajan seuranta Arttu.xlsx
+++ b/docs/Työajan seuranta Arttu.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juhaj\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arttu\Dropbox\Koulu\Web-ohjelmoinnin sovellusprojekti\Movieproject\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DB270A96-4B16-40E8-9C51-6444C08D5D7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AAE3B16-7C17-43F4-B88D-05535A758A59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1425" yWindow="1425" windowWidth="21600" windowHeight="11835" xr2:uid="{B7036960-D674-4B76-B564-D076AACD5E6B}"/>
+    <workbookView xWindow="12045" yWindow="6255" windowWidth="17670" windowHeight="9870" xr2:uid="{B7036960-D674-4B76-B564-D076AACD5E6B}"/>
   </bookViews>
   <sheets>
     <sheet name="Arttu Jämsä" sheetId="3" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>Ryhmä:</t>
   </si>
@@ -78,6 +78,18 @@
   </si>
   <si>
     <t>Review API create &amp; search</t>
+  </si>
+  <si>
+    <t>24.9.</t>
+  </si>
+  <si>
+    <t>Review API update, delete ja testit</t>
+  </si>
+  <si>
+    <t>26.9.</t>
+  </si>
+  <si>
+    <t>koodin korjausta ehdotusten mukaiseksi</t>
   </si>
 </sst>
 </file>
@@ -433,7 +445,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C1EECD9-4AD3-41AF-8923-B28678799497}">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.85546875" customWidth="1"/>
@@ -515,12 +527,42 @@
         <v>3.5</v>
       </c>
     </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="44038759-07ae-40d4-bc3d-7c9fb0b3775b" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009BAF6AFB37B6774A9122C6036818BC92" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c611cd0fe7e35dfe638a44e659100205">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="44038759-07ae-40d4-bc3d-7c9fb0b3775b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="36a43d4c38ea7f7b42b5de64d2c1c906" ns3:_="">
     <xsd:import namespace="44038759-07ae-40d4-bc3d-7c9fb0b3775b"/>
@@ -700,14 +742,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="44038759-07ae-40d4-bc3d-7c9fb0b3775b" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -718,6 +752,16 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3DBD177-6275-4D31-B82C-61F9284D9B7B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="44038759-07ae-40d4-bc3d-7c9fb0b3775b"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B52374CD-1656-483C-BC7A-A879F7105755}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -735,16 +779,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3DBD177-6275-4D31-B82C-61F9284D9B7B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="44038759-07ae-40d4-bc3d-7c9fb0b3775b"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{28C42445-4535-4827-89B5-92D7D04A90E8}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Group Join frontend started and bugging out
</commit_message>
<xml_diff>
--- a/docs/Työajan seuranta Arttu.xlsx
+++ b/docs/Työajan seuranta Arttu.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arttu\Dropbox\Koulu\Web-ohjelmoinnin sovellusprojekti\Movieproject\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FEC8A8C-AAFC-4B53-8D57-74FEC53A3C34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{054D71BA-0C1C-4DC2-8CEE-C0CFCCBC85D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="4740" yWindow="6870" windowWidth="17670" windowHeight="9870" xr2:uid="{B7036960-D674-4B76-B564-D076AACD5E6B}"/>
+    <workbookView xWindow="3345" yWindow="5955" windowWidth="17670" windowHeight="9870" xr2:uid="{B7036960-D674-4B76-B564-D076AACD5E6B}"/>
   </bookViews>
   <sheets>
     <sheet name="Arttu Jämsä" sheetId="3" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>Ryhmä:</t>
   </si>
@@ -96,6 +96,12 @@
   </si>
   <si>
     <t>Group Join API tekoa</t>
+  </si>
+  <si>
+    <t>1.10.</t>
+  </si>
+  <si>
+    <t>Group Join frontendia</t>
   </si>
 </sst>
 </file>
@@ -451,7 +457,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C1EECD9-4AD3-41AF-8923-B28678799497}">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.85546875" customWidth="1"/>
@@ -566,20 +572,23 @@
         <v>3.5</v>
       </c>
     </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11">
+        <v>3.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="44038759-07ae-40d4-bc3d-7c9fb0b3775b" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009BAF6AFB37B6774A9122C6036818BC92" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c611cd0fe7e35dfe638a44e659100205">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="44038759-07ae-40d4-bc3d-7c9fb0b3775b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="36a43d4c38ea7f7b42b5de64d2c1c906" ns3:_="">
     <xsd:import namespace="44038759-07ae-40d4-bc3d-7c9fb0b3775b"/>
@@ -759,6 +768,14 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="44038759-07ae-40d4-bc3d-7c9fb0b3775b" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -769,16 +786,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3DBD177-6275-4D31-B82C-61F9284D9B7B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="44038759-07ae-40d4-bc3d-7c9fb0b3775b"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B52374CD-1656-483C-BC7A-A879F7105755}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -796,6 +803,16 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3DBD177-6275-4D31-B82C-61F9284D9B7B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="44038759-07ae-40d4-bc3d-7c9fb0b3775b"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{28C42445-4535-4827-89B5-92D7D04A90E8}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Navbar visuals and remove member error handling improved. Owner cannot remove remove themselves check added to backend
</commit_message>
<xml_diff>
--- a/docs/Työajan seuranta Arttu.xlsx
+++ b/docs/Työajan seuranta Arttu.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arttu\Dropbox\Koulu\Web-ohjelmoinnin sovellusprojekti\Movieproject\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FC2A20B-E118-46B8-A0D5-50ACA2D287F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DE6E3FC-D88B-42D6-BAE1-C27C789B32DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3345" yWindow="5955" windowWidth="17670" windowHeight="9870" xr2:uid="{B7036960-D674-4B76-B564-D076AACD5E6B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>Ryhmä:</t>
   </si>
@@ -120,6 +120,12 @@
   </si>
   <si>
     <t>Manuaali merge, bugien poistaminen ja muutosehdotusten implementointi</t>
+  </si>
+  <si>
+    <t>5.10.</t>
+  </si>
+  <si>
+    <t>Group member removal</t>
   </si>
 </sst>
 </file>
@@ -475,7 +481,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C1EECD9-4AD3-41AF-8923-B28678799497}">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.85546875" customWidth="1"/>
@@ -634,12 +640,40 @@
         <v>2</v>
       </c>
     </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15">
+        <v>2.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="44038759-07ae-40d4-bc3d-7c9fb0b3775b" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009BAF6AFB37B6774A9122C6036818BC92" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c611cd0fe7e35dfe638a44e659100205">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="44038759-07ae-40d4-bc3d-7c9fb0b3775b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="36a43d4c38ea7f7b42b5de64d2c1c906" ns3:_="">
     <xsd:import namespace="44038759-07ae-40d4-bc3d-7c9fb0b3775b"/>
@@ -819,24 +853,25 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="44038759-07ae-40d4-bc3d-7c9fb0b3775b" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{28C42445-4535-4827-89B5-92D7D04A90E8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3DBD177-6275-4D31-B82C-61F9284D9B7B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="44038759-07ae-40d4-bc3d-7c9fb0b3775b"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B52374CD-1656-483C-BC7A-A879F7105755}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -854,24 +889,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3DBD177-6275-4D31-B82C-61F9284D9B7B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="44038759-07ae-40d4-bc3d-7c9fb0b3775b"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{28C42445-4535-4827-89B5-92D7D04A90E8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{9f9ce49a-5101-4aa3-8c75-0d5935ad6525}" enabled="0" method="" siteId="{9f9ce49a-5101-4aa3-8c75-0d5935ad6525}" removed="1"/>

</xml_diff>

<commit_message>
Added few api endpoints
</commit_message>
<xml_diff>
--- a/docs/Työajan seuranta Arttu.xlsx
+++ b/docs/Työajan seuranta Arttu.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arttu\Dropbox\Koulu\Web-ohjelmoinnin sovellusprojekti\Movieproject\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69D9855F-8668-4956-9432-724A092C118D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8CF97B3-FF67-48B5-A7F5-F9FDD9B6EDE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14895" yWindow="6900" windowWidth="17670" windowHeight="9870" xr2:uid="{B7036960-D674-4B76-B564-D076AACD5E6B}"/>
+    <workbookView xWindow="3345" yWindow="5955" windowWidth="17670" windowHeight="9870" xr2:uid="{B7036960-D674-4B76-B564-D076AACD5E6B}"/>
   </bookViews>
   <sheets>
     <sheet name="Arttu Jämsä" sheetId="3" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
   <si>
     <t>Ryhmä:</t>
   </si>
@@ -138,6 +138,18 @@
   </si>
   <si>
     <t>Leave group ja change owner</t>
+  </si>
+  <si>
+    <t>8.10.</t>
+  </si>
+  <si>
+    <t>Implementing suggested fixes</t>
+  </si>
+  <si>
+    <t>9.10.</t>
+  </si>
+  <si>
+    <t>API dokumentaation lisäystä, PR arviointia</t>
   </si>
 </sst>
 </file>
@@ -493,7 +505,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C1EECD9-4AD3-41AF-8923-B28678799497}">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.85546875" customWidth="1"/>
@@ -685,12 +697,42 @@
         <v>4</v>
       </c>
     </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>34</v>
+      </c>
+      <c r="B18" t="s">
+        <v>35</v>
+      </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19" t="s">
+        <v>37</v>
+      </c>
+      <c r="C19">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="44038759-07ae-40d4-bc3d-7c9fb0b3775b" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009BAF6AFB37B6774A9122C6036818BC92" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c611cd0fe7e35dfe638a44e659100205">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="44038759-07ae-40d4-bc3d-7c9fb0b3775b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="36a43d4c38ea7f7b42b5de64d2c1c906" ns3:_="">
     <xsd:import namespace="44038759-07ae-40d4-bc3d-7c9fb0b3775b"/>
@@ -870,7 +912,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -879,15 +921,17 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="44038759-07ae-40d4-bc3d-7c9fb0b3775b" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3DBD177-6275-4D31-B82C-61F9284D9B7B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="44038759-07ae-40d4-bc3d-7c9fb0b3775b"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B52374CD-1656-483C-BC7A-A879F7105755}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -905,7 +949,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{28C42445-4535-4827-89B5-92D7D04A90E8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -913,16 +957,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3DBD177-6275-4D31-B82C-61F9284D9B7B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="44038759-07ae-40d4-bc3d-7c9fb0b3775b"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{9f9ce49a-5101-4aa3-8c75-0d5935ad6525}" enabled="0" method="" siteId="{9f9ce49a-5101-4aa3-8c75-0d5935ad6525}" removed="1"/>

</xml_diff>